<commit_message>
Remove company name from quotation template
</commit_message>
<xml_diff>
--- a/plugins/quotation-maker/skills/create-quotation/assets/系统报价单模板.xlsx
+++ b/plugins/quotation-maker/skills/create-quotation/assets/系统报价单模板.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="19">
   <si>
-    <t>洋流科技有限公司</t>
+    <t/>
   </si>
   <si>
     <t>服务内容</t>
@@ -1488,9 +1488,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
+      <c r="A1" s="3"/>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>

</xml_diff>